<commit_message>
Auto update CodeMetrix trackers
</commit_message>
<xml_diff>
--- a/Students.xlsx
+++ b/Students.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Students" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Students'!$A$1:$E$360</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Students'!$A$1:$E$361</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E360"/>
+  <dimension ref="A1:E361"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -467,17 +467,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>922525106263</t>
+          <t>922525106269</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>RUBESH C</t>
+          <t>Sakthivel. M</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Rubesh_7</t>
+          <t>sakthivel23116</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -487,24 +487,24 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/Rubesh_7/</t>
+          <t>https://leetcode.com/u/sakthivel23116/</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>922525106283</t>
+          <t>922525106275</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>SANTHOSH S</t>
+          <t>SANJAY U</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>SanthoshSathya260</t>
+          <t>SanjayUdayan</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -514,24 +514,24 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/SanthoshSathya260/</t>
+          <t>https://leetcode.com/u/SanjayUdayan/</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>922525106291</t>
+          <t>922525106283</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>SARVESWARAN R</t>
+          <t>SANTHOSH S</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>sarvesh312008</t>
+          <t>SanthoshSathya260</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -541,24 +541,24 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/sarvesh312008/</t>
+          <t>https://leetcode.com/u/SanthoshSathya260/</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>922525106292</t>
+          <t>922525106291</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>SASHMIKA.P</t>
+          <t>SARVESWARAN R</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>sashmikaprabhu</t>
+          <t>sarvesh312008</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -568,24 +568,24 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/sashmikaprabhu/</t>
+          <t>https://leetcode.com/u/sarvesh312008/</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>922525106307</t>
+          <t>922525106292</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>SHIVANI B</t>
+          <t>SASHMIKA.P</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>shivani208</t>
+          <t>sashmikaprabhu</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -595,24 +595,24 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/shivani208/</t>
+          <t>https://leetcode.com/u/sashmikaprabhu/</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>922525106272</t>
+          <t>922525106307</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>SANJAY D</t>
+          <t>SHIVANI B</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>itsmesanjay007</t>
+          <t>shivani208</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -622,24 +622,24 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/itsmesanjay007/</t>
+          <t>https://leetcode.com/u/shivani208/</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>922525106309</t>
+          <t>922525106272</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>SHREE CHARAN T</t>
+          <t>SANJAY D</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>shreecharan22</t>
+          <t>itsmesanjay007</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -649,24 +649,24 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/shreecharan22/</t>
+          <t>https://leetcode.com/u/itsmesanjay007/</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>922525106314</t>
+          <t>922525106309</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>SIVANESH D</t>
+          <t>SHREE CHARAN T</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>sivanesh2007</t>
+          <t>shreecharan22</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -676,24 +676,24 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/sivanesh2007/</t>
+          <t>https://leetcode.com/u/shreecharan22/</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>922525196293</t>
+          <t>922525106314</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>SASWIN D</t>
+          <t>SIVANESH D</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>saswin_88</t>
+          <t>sivanesh2007</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -703,24 +703,24 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/saswin_88/</t>
+          <t>https://leetcode.com/u/sivanesh2007/</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>922525106253</t>
+          <t>922525196293</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>RITHANYA KN</t>
+          <t>SASWIN D</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Rithanya12-3</t>
+          <t>saswin_88</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -730,24 +730,24 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/Rithanya12-3/</t>
+          <t>https://leetcode.com/u/saswin_88/</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>922525106257</t>
+          <t>922525106264</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>RITHIKA B</t>
+          <t>SABAREESH K</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Rithika_Balakrishnan</t>
+          <t>sabareesh_karikalan</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -757,24 +757,24 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/Rithika_Balakrishnan/</t>
+          <t>https://leetcode.com/u/sabareesh_karikalan/</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>922525106259</t>
+          <t>922525106253</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>ROHITH V</t>
+          <t>RITHANYA KN</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>RohithrohiV</t>
+          <t>Rithanya12-3</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -784,24 +784,24 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/RohithrohiV/</t>
+          <t>https://leetcode.com/u/Rithanya12-3/</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>922525106260</t>
+          <t>922525106257</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ROOBAGAPRIYA R</t>
+          <t>RITHIKA B</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Roobagapriya</t>
+          <t>Rithika_Balakrishnan</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -811,24 +811,24 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/Roobagapriya/</t>
+          <t>https://leetcode.com/u/Rithika_Balakrishnan/</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>922525106256</t>
+          <t>922525106259</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>RITHIK P</t>
+          <t>ROHITH V</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Rithik_78</t>
+          <t>RohithrohiV</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -838,24 +838,24 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/Rithik_78/</t>
+          <t>https://leetcode.com/u/RohithrohiV/</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>922525106258</t>
+          <t>922525106256</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>RITHISH R</t>
+          <t>RITHIK P</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Rithish_</t>
+          <t>Rithik_78</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -865,24 +865,24 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/Rithish_/</t>
+          <t>https://leetcode.com/u/Rithik_78/</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>922525106264</t>
+          <t>922525106258</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>SABAREESH K</t>
+          <t>RITHISH R</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>sabareesh_karikalan</t>
+          <t>Rithish_</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -892,24 +892,24 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/sabareesh_karikalan/</t>
+          <t>https://leetcode.com/u/Rithish_/</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>922525106266</t>
+          <t>922525106260</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>SAHANA.V</t>
+          <t>ROOBAGAPRIYA R</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Sahanavijayakumar_0033</t>
+          <t>Roobagapriya</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -919,24 +919,24 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/Sahanavijayakumar_0033/</t>
+          <t>https://leetcode.com/u/Roobagapriya/</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>922525106269</t>
+          <t>922525106266</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Sakthivel. M</t>
+          <t>SAHANA.V</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>sakthivel23116</t>
+          <t>Sahanavijayakumar_0033</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -946,7 +946,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/sakthivel23116/</t>
+          <t>https://leetcode.com/u/Sahanavijayakumar_0033/</t>
         </is>
       </c>
     </row>
@@ -1007,17 +1007,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>922525106275</t>
+          <t>922525106263</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>SANJAY U</t>
+          <t>RUBESH C</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>SanjayUdayan</t>
+          <t>Rubesh_7</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1027,7 +1027,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/SanjayUdayan/</t>
+          <t>https://leetcode.com/u/Rubesh_7/</t>
         </is>
       </c>
     </row>
@@ -1844,17 +1844,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>922525106367</t>
+          <t>922525106365</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>VIKRAM V</t>
+          <t>VIGNESHWAR U</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>vikramvicky5678</t>
+          <t>VIGNESHWAR0221</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -1864,24 +1864,24 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/vikramvicky5678/</t>
+          <t>https://leetcode.com/u/VIGNESHWAR0221/</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>922525106368</t>
+          <t>922525106366</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>VISHNU B</t>
+          <t>VIJAYARAGAVAN R</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>VISHNU_B_2008</t>
+          <t>vijayaragavan1216</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -1891,24 +1891,24 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/VISHNU_B_2008/</t>
+          <t>https://leetcode.com/u/vijayaragavan1216/</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>922525106369</t>
+          <t>922525106367</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>VISHNU PRIYAN S</t>
+          <t>VIKRAM V</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>itz__priyan__</t>
+          <t>vikramvicky5678</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -1918,24 +1918,24 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/itz__priyan__/</t>
+          <t>https://leetcode.com/u/vikramvicky5678/</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>922525106370</t>
+          <t>922525106368</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>VISHNUHARAN V S</t>
+          <t>VISHNU B</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Vishnuharan082007</t>
+          <t>VISHNU_B_2008</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -1945,24 +1945,24 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/Vishnuharan082007/</t>
+          <t>https://leetcode.com/u/VISHNU_B_2008/</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>922525106365</t>
+          <t>922525106369</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>VIGNESHWAR U</t>
+          <t>VISHNU PRIYAN S</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>VIGNESHWAR0221</t>
+          <t>itz__priyan__</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -1972,24 +1972,24 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/VIGNESHWAR0221/</t>
+          <t>https://leetcode.com/u/itz__priyan__/</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>922525106359</t>
+          <t>922525106362</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>VASANTHKUMAR R</t>
+          <t>VELLIANGIRI R</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>VasanthKumar008</t>
+          <t>velliangiri_R</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -1999,24 +1999,24 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/VasanthKumar008/</t>
+          <t>https://leetcode.com/u/velliangiri_R/</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>922525106360</t>
+          <t>922525106357</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>VASUDEVAN G</t>
+          <t>VASANTH S</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>GTVASU2008</t>
+          <t>_vasanth_s_</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -2026,24 +2026,24 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/GTVASU2008/</t>
+          <t>https://leetcode.com/u/_vasanth_s_/</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>922525106361</t>
+          <t>922525106358</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>VASUKI K</t>
+          <t>VASANTHA KUMAR D</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>vasuki</t>
+          <t>Vasanthakumar12232</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -2053,24 +2053,24 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/vasuki/</t>
+          <t>https://leetcode.com/u/Vasanthakumar12232/</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>922525106362</t>
+          <t>922525106359</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>VELLIANGIRI R</t>
+          <t>VASANTHKUMAR R</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>velliangiri_R</t>
+          <t>VasanthKumar008</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -2080,24 +2080,24 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/velliangiri_R/</t>
+          <t>https://leetcode.com/u/VasanthKumar008/</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>922525106363</t>
+          <t>922525106360</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>VIGNESH M</t>
+          <t>VASUDEVAN G</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>O8bYDSRUbE</t>
+          <t>GTVASU2008</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -2107,24 +2107,24 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/O8bYDSRUbE/</t>
+          <t>https://leetcode.com/u/GTVASU2008/</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>922525106366</t>
+          <t>922525106361</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>VIJAYARAGAVAN R</t>
+          <t>VASUKI K</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>vijayaragavan1216</t>
+          <t>vasuki</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -2134,24 +2134,24 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/vijayaragavan1216/</t>
+          <t>https://leetcode.com/u/vasuki/</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>922525106371</t>
+          <t>922525106363</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>VISHNUPRIYA S</t>
+          <t>VIGNESH M</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>vishnupriyamaran</t>
+          <t>O8bYDSRUbE</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -2161,24 +2161,24 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/vishnupriyamaran/</t>
+          <t>https://leetcode.com/u/O8bYDSRUbE/</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>922525106372</t>
+          <t>922525106370</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>VISHWAJETH A M</t>
+          <t>VISHNUHARAN V S</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>vishwajeth</t>
+          <t>Vishnuharan082007</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -2188,24 +2188,24 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/vishwajeth/</t>
+          <t>https://leetcode.com/u/Vishnuharan082007/</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>922525106373</t>
+          <t>922525106371</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>YASHNI S</t>
+          <t>VISHNUPRIYA S</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Yashnisubramaniyan</t>
+          <t>vishnupriyamaran</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -2215,24 +2215,24 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/Yashnisubramaniyan/</t>
+          <t>https://leetcode.com/u/vishnupriyamaran/</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>922525106374</t>
+          <t>922525106372</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>YASWANTH V</t>
+          <t>VISHWAJETH A M</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>yaswanth_2008</t>
+          <t>vishwajeth</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -2242,24 +2242,24 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/yaswanth_2008/</t>
+          <t>https://leetcode.com/u/vishwajeth/</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>922525106375</t>
+          <t>922525106373</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>YAZHINI M</t>
+          <t>YASHNI S</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>yazhini2007</t>
+          <t>Yashnisubramaniyan</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -2269,24 +2269,24 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/yazhini2007/</t>
+          <t>https://leetcode.com/u/Yashnisubramaniyan/</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>922525106376</t>
+          <t>922525106374</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>YAZHINI S</t>
+          <t>YASWANTH V</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>yazhini__1234</t>
+          <t>yaswanth_2008</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -2296,24 +2296,24 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/yazhini__1234/</t>
+          <t>https://leetcode.com/u/yaswanth_2008/</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>922525106316</t>
+          <t>922525106375</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>SIVARANJAN M P</t>
+          <t>YAZHINI M</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>SIVARANJAN_MP</t>
+          <t>yazhini2007</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -2323,24 +2323,24 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/SIVARANJAN_MP/</t>
+          <t>https://leetcode.com/u/yazhini2007/</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>922525106317</t>
+          <t>922525106316</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>SIVASANJEEV P</t>
+          <t>SIVARANJAN M P</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Sivasanjeev16</t>
+          <t>SIVARANJAN_MP</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -2350,24 +2350,24 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/Sivasanjeev16/</t>
+          <t>https://leetcode.com/u/SIVARANJAN_MP/</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>922525106318</t>
+          <t>922525106317</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>SIVASUBRAMANI A</t>
+          <t>SIVASANJEEV P</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>AK_Siva</t>
+          <t>Sivasanjeev16</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -2377,24 +2377,24 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/AK_Siva/</t>
+          <t>https://leetcode.com/u/Sivasanjeev16/</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>922525106319</t>
+          <t>922525106318</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>SIVATHARUN C</t>
+          <t>SIVASUBRAMANI A</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>sivatharun22</t>
+          <t>AK_Siva</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -2404,24 +2404,24 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/sivatharun22/</t>
+          <t>https://leetcode.com/u/AK_Siva/</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>922525106320</t>
+          <t>922525106319</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>SOBIKA R</t>
+          <t>SIVATHARUN C</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>_sobika_R</t>
+          <t>sivatharun22</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -2431,24 +2431,24 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/_sobika_R/</t>
+          <t>https://leetcode.com/u/sivatharun22/</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>922525106321</t>
+          <t>922525106320</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>SREE DHARANI C</t>
+          <t>SOBIKA R</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>SREEDHARANI_14</t>
+          <t>_sobika_R</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -2458,24 +2458,24 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/SREEDHARANI_14/</t>
+          <t>https://leetcode.com/u/_sobika_R/</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>922525106322</t>
+          <t>922525106321</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>SRI  T</t>
+          <t>SREE DHARANI C</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Sri1540</t>
+          <t>SREEDHARANI_14</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -2485,24 +2485,24 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/Sri1540/</t>
+          <t>https://leetcode.com/u/SREEDHARANI_14/</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>922525106323</t>
+          <t>922525106322</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>SRI HEERA J</t>
+          <t>SRI  T</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>sriheera03</t>
+          <t>Sri1540</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -2512,24 +2512,24 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/sriheera03/</t>
+          <t>https://leetcode.com/u/Sri1540/</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>922525106324</t>
+          <t>922525106323</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>SRI KANTH R</t>
+          <t>SRI HEERA J</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>kanth2008</t>
+          <t>sriheera03</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -2539,24 +2539,24 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/kanth2008/</t>
+          <t>https://leetcode.com/u/sriheera03/</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>922525106325</t>
+          <t>922525106324</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>SRI SASTIKA G</t>
+          <t>SRI KANTH R</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Srisastika_1401</t>
+          <t>kanth2008</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -2566,24 +2566,24 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/Srisastika_1401/</t>
+          <t>https://leetcode.com/u/kanth2008/</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>922525106326</t>
+          <t>922525106325</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>SRI VARSHAN B P</t>
+          <t>SRI SASTIKA G</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>srivarshan_B_P</t>
+          <t>Srisastika_1401</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -2593,24 +2593,24 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/srivarshan_B_P/</t>
+          <t>https://leetcode.com/u/Srisastika_1401/</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>922525106327</t>
+          <t>922525106326</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>SRINATH V</t>
+          <t>SRI VARSHAN B P</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>V_SRINATH</t>
+          <t>srivarshan_B_P</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -2620,24 +2620,24 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/V_SRINATH/</t>
+          <t>https://leetcode.com/u/srivarshan_B_P/</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>922525106328</t>
+          <t>922525106327</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>SRINIRANJAN S</t>
+          <t>SRINATH V</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>SRINIRANJAN2008</t>
+          <t>V_SRINATH</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -2647,24 +2647,24 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/SRINIRANJAN2008/</t>
+          <t>https://leetcode.com/u/V_SRINATH/</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>922525106329</t>
+          <t>922525106328</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>SRINITHE T</t>
+          <t>SRINIRANJAN S</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>srinithe_1401</t>
+          <t>SRINIRANJAN2008</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -2674,24 +2674,24 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/srinithe_1401/</t>
+          <t>https://leetcode.com/u/SRINIRANJAN2008/</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>922525106364</t>
+          <t>922525106329</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>VIGNESH VELAN M</t>
+          <t>SRINITHE T</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Vicky_27_Velan</t>
+          <t>srinithe_1401</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -2701,7 +2701,7 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/Vicky_27_Velan/</t>
+          <t>https://leetcode.com/u/srinithe_1401/</t>
         </is>
       </c>
     </row>
@@ -2762,17 +2762,17 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>922525106378</t>
+          <t>922525106376</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>YOKESWARAN S</t>
+          <t>YAZHINI S</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>syokeswaran</t>
+          <t>yazhini__1234</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -2782,24 +2782,24 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/syokeswaran/</t>
+          <t>https://leetcode.com/u/yazhini__1234/</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>922525106330</t>
+          <t>922525106378</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>SRINITHI S</t>
+          <t>YOKESWARAN S</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Srinithi24_</t>
+          <t>syokeswaran</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -2809,24 +2809,24 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/Srinithi24_/</t>
+          <t>https://leetcode.com/u/syokeswaran/</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>922525106339</t>
+          <t>922525106330</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>SUJITH RAJA B</t>
+          <t>SRINITHI S</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>mahi20_</t>
+          <t>Srinithi24_</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -2836,24 +2836,24 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/mahi20_/</t>
+          <t>https://leetcode.com/u/Srinithi24_/</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>922525106353</t>
+          <t>922525106339</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>THIRISHA C</t>
+          <t>SUJITH RAJA B</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>thirishavsb</t>
+          <t>mahi20_</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -2863,24 +2863,24 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/thirishavsb/</t>
+          <t>https://leetcode.com/u/mahi20_/</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>922525106331</t>
+          <t>922525106353</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>SRISAMAYA R</t>
+          <t>THIRISHA C</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>mahi</t>
+          <t>thirishavsb</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -2890,24 +2890,24 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/mahi/</t>
+          <t>https://leetcode.com/u/thirishavsb/</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>922525106332</t>
+          <t>922525106331</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>SUBARNA V</t>
+          <t>SRISAMAYA R</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Subarna_17</t>
+          <t>mahi</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -2917,24 +2917,24 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/Subarna_17/</t>
+          <t>https://leetcode.com/u/mahi/</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>922525106334</t>
+          <t>922525106364</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>SUBIKA T</t>
+          <t>VIGNESH VELAN M</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>subika1112</t>
+          <t>Vicky_27_Velan</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -2944,24 +2944,24 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/subika1112/</t>
+          <t>https://leetcode.com/u/Vicky_27_Velan/</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>922525106335</t>
+          <t>922525106332</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>SUDHARSAN S</t>
+          <t>SUBARNA V</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Sudharsan</t>
+          <t>Subarna_17</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -2971,24 +2971,24 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/Sudharsan/</t>
+          <t>https://leetcode.com/u/Subarna_17/</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>922525106336</t>
+          <t>922525106334</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>SUGANTHAN K</t>
+          <t>SUBIKA T</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>SUGANTHKALAI</t>
+          <t>subika1112</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -2998,24 +2998,24 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/SUGANTHKALAI/</t>
+          <t>https://leetcode.com/u/subika1112/</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>922525106337</t>
+          <t>922525106335</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>SUGIDHARSHINI T</t>
+          <t>SUDHARSAN S</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Sugi_07</t>
+          <t>Sudharsan</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -3025,24 +3025,24 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/Sugi_07/</t>
+          <t>https://leetcode.com/u/Sudharsan/</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>922525106338</t>
+          <t>922525106336</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>SUJEETH M</t>
+          <t>SUGANTHAN K</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>SUJEETH77</t>
+          <t>SUGANTHKALAI</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -3052,24 +3052,24 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/SUJEETH77/</t>
+          <t>https://leetcode.com/u/SUGANTHKALAI/</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>922525106340</t>
+          <t>922525106337</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>SUMITHRA S</t>
+          <t>SUGIDHARSHINI T</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>sumithra_16</t>
+          <t>Sugi_07</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -3079,24 +3079,24 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/sumithra_16/</t>
+          <t>https://leetcode.com/u/Sugi_07/</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>922525106341</t>
+          <t>922525106338</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>SURYA PRABHU S</t>
+          <t>SUJEETH M</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>surya001prabhu</t>
+          <t>SUJEETH77</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -3106,24 +3106,24 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/surya001prabhu/</t>
+          <t>https://leetcode.com/u/SUJEETH77/</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>922525106342</t>
+          <t>922525106340</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>SUSIDHARAN M</t>
+          <t>SUMITHRA S</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Susidharan147</t>
+          <t>sumithra_16</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -3133,24 +3133,24 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/Susidharan147/</t>
+          <t>https://leetcode.com/u/sumithra_16/</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>922525106343</t>
+          <t>922525106341</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>SUTHARSHANA S</t>
+          <t>SURYA PRABHU S</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>sutharshana743</t>
+          <t>surya001prabhu</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -3160,24 +3160,24 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/sutharshana743/</t>
+          <t>https://leetcode.com/u/surya001prabhu/</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>922525106344</t>
+          <t>922525106342</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>SWATHI M</t>
+          <t>SUSIDHARAN M</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Swathimanivel_1234</t>
+          <t>Susidharan147</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -3187,24 +3187,24 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/Swathimanivel_1234/</t>
+          <t>https://leetcode.com/u/Susidharan147/</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>922525106345</t>
+          <t>922525106343</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>SWATHI S</t>
+          <t>SUTHARSHANA S</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>_swathi _3366</t>
+          <t>sutharshana743</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -3214,24 +3214,24 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/_swathi _3366/</t>
+          <t>https://leetcode.com/u/sutharshana743/</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>922525106347</t>
+          <t>922525106344</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>TAMIL SELVAN R</t>
+          <t>SWATHI M</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Kdmif0HMNm</t>
+          <t>Swathimanivel_1234</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -3241,24 +3241,24 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/Kdmif0HMNm/</t>
+          <t>https://leetcode.com/u/Swathimanivel_1234/</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>922525106348</t>
+          <t>922525106345</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>THAMARAI SELVI D</t>
+          <t>SWATHI S</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>thamarai_04</t>
+          <t>_swathi _3366</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -3268,24 +3268,24 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/thamarai_04/</t>
+          <t>https://leetcode.com/u/_swathi _3366/</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>922525106349</t>
+          <t>922525106347</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>THAMEEM FARSHITHA A</t>
+          <t>TAMIL SELVAN R</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Thameem_786</t>
+          <t>Kdmif0HMNm</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -3295,24 +3295,24 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/Thameem_786/</t>
+          <t>https://leetcode.com/u/Kdmif0HMNm/</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>922525106350</t>
+          <t>922525106348</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>THARANISH R</t>
+          <t>THAMARAI SELVI D</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>THARANISH2008</t>
+          <t>thamarai_04</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -3322,24 +3322,24 @@
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/THARANISH2008/</t>
+          <t>https://leetcode.com/u/thamarai_04/</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>922525106351</t>
+          <t>922525106349</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>THARUNIKA P</t>
+          <t>THAMEEM FARSHITHA A</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Tharunika_12</t>
+          <t>Thameem_786</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -3349,24 +3349,24 @@
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/Tharunika_12/</t>
+          <t>https://leetcode.com/u/Thameem_786/</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>922525106352</t>
+          <t>922525106350</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>THIRINESH KUMAR S</t>
+          <t>THARANISH R</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>THIRINESH KUMAR.S</t>
+          <t>THARANISH2008</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -3376,24 +3376,24 @@
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/THIRINESH KUMAR.S/</t>
+          <t>https://leetcode.com/u/THARANISH2008/</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>922525106354</t>
+          <t>922525106351</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>THIRUMURUGAN S</t>
+          <t>THARUNIKA P</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>thiru0211_</t>
+          <t>Tharunika_12</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -3403,24 +3403,24 @@
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/thiru0211_/</t>
+          <t>https://leetcode.com/u/Tharunika_12/</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>922525106355</t>
+          <t>922525106352</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>VAISHNAVI U</t>
+          <t>THIRINESH KUMAR S</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>vaish200</t>
+          <t>THIRINESH KUMAR.S</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -3430,24 +3430,24 @@
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/vaish200/</t>
+          <t>https://leetcode.com/u/THIRINESH KUMAR.S/</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>922525106356</t>
+          <t>922525106354</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>VASANTH KUMAR C</t>
+          <t>THIRUMURUGAN S</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>VASANTH2007</t>
+          <t>thiru0211_</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -3457,24 +3457,24 @@
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/VASANTH2007/</t>
+          <t>https://leetcode.com/u/thiru0211_/</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>922525106357</t>
+          <t>922525106355</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>VASANTH S</t>
+          <t>VAISHNAVI U</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>_vasanth_s_</t>
+          <t>vaish200</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -3484,24 +3484,24 @@
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/_vasanth_s_/</t>
+          <t>https://leetcode.com/u/vaish200/</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>922525106358</t>
+          <t>922525106356</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>VASANTHA KUMAR D</t>
+          <t>VASANTH KUMAR C</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Vasanthakumar12232</t>
+          <t>VASANTH2007</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -3511,7 +3511,7 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/Vasanthakumar12232/</t>
+          <t>https://leetcode.com/u/VASANTH2007/</t>
         </is>
       </c>
     </row>
@@ -6110,17 +6110,17 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>922525106027</t>
+          <t>922525106008</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>Arulesh K</t>
+          <t>AHELESH G S</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>arul2008</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D211" t="inlineStr">
@@ -6130,7 +6130,7 @@
       </c>
       <c r="E211" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/arul2008/</t>
+          <t>https://leetcode.com/u/B/</t>
         </is>
       </c>
     </row>
@@ -6893,17 +6893,17 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>922525106008</t>
+          <t>922525106027</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>AHELESH G S</t>
+          <t>Arulesh K</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>arul2008</t>
         </is>
       </c>
       <c r="D240" t="inlineStr">
@@ -6913,7 +6913,7 @@
       </c>
       <c r="E240" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/B/</t>
+          <t>https://leetcode.com/u/arul2008/</t>
         </is>
       </c>
     </row>
@@ -10157,8 +10157,35 @@
         </is>
       </c>
     </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>922525106381</t>
+        </is>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>LOHITH T S</t>
+        </is>
+      </c>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>LOHITH206</t>
+        </is>
+      </c>
+      <c r="D361" t="inlineStr">
+        <is>
+          <t>ECE E</t>
+        </is>
+      </c>
+      <c r="E361" t="inlineStr">
+        <is>
+          <t>https://leetcode.com/u/LOHITH206/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E360"/>
+  <autoFilter ref="A1:E361"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update tracker data files, history, and student rosters
</commit_message>
<xml_diff>
--- a/Students.xlsx
+++ b/Students.xlsx
@@ -1223,17 +1223,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>922525106280</t>
+          <t>922525106284</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>SANTHOSH D</t>
+          <t>Santhosh S</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>santhosh7811</t>
+          <t>santhosh2407</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1243,24 +1243,24 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/santhosh7811/</t>
+          <t>https://leetcode.com/u/santhosh2407/</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>922525106284</t>
+          <t>922525106285</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Santhosh S</t>
+          <t>SANTHOSH V</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>santhosh2407</t>
+          <t>santhosh8760</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1270,24 +1270,24 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/santhosh2407/</t>
+          <t>https://leetcode.com/u/santhosh8760/</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>922525106285</t>
+          <t>922525106286</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>SANTHOSH V</t>
+          <t>SARAN K</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>santhosh8760</t>
+          <t>saran32</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1297,24 +1297,24 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/santhosh8760/</t>
+          <t>https://leetcode.com/u/saran32/</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>922525106286</t>
+          <t>922525106288</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>SARAN K</t>
+          <t>SARAVANAN K</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>saran32</t>
+          <t>saravanan__k__</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1324,24 +1324,24 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/saran32/</t>
+          <t>https://leetcode.com/u/saravanan__k__/</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>922525106288</t>
+          <t>922525106289</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>SARAVANAN K</t>
+          <t>SARAVANAN S</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>saravanan__k__</t>
+          <t>Saravanan_7525</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1351,24 +1351,24 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/saravanan__k__/</t>
+          <t>https://leetcode.com/u/Saravanan_7525/</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>922525106289</t>
+          <t>922525106290</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>SARAVANAN S</t>
+          <t>SARIKA M P</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Saravanan_7525</t>
+          <t>sarika_5408</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1378,24 +1378,24 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/Saravanan_7525/</t>
+          <t>https://leetcode.com/u/sarika_5408/</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>922525106290</t>
+          <t>922525106296</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>SARIKA M P</t>
+          <t>SELVAKUMAR K</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>sarika_5408</t>
+          <t>Selvakumarsk-32</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1405,24 +1405,24 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/sarika_5408/</t>
+          <t>https://leetcode.com/u/Selvakumarsk-32/</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>922525106296</t>
+          <t>922525106297</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>SELVAKUMAR K</t>
+          <t>SELVAPRAGADEESH S</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Selvakumarsk-32</t>
+          <t>Selvapragadeesh</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1432,24 +1432,24 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/Selvakumarsk-32/</t>
+          <t>https://leetcode.com/u/Selvapragadeesh/</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>922525106297</t>
+          <t>922525106298</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>SELVAPRAGADEESH S</t>
+          <t>SELVA RAGAVAN</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Selvapragadeesh</t>
+          <t>Selvax07</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1459,24 +1459,24 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/Selvapragadeesh/</t>
+          <t>https://leetcode.com/u/Selvax07/</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>922525106298</t>
+          <t>922525106299</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>SELVA RAGAVAN</t>
+          <t>SENTHAMIZHSELVAN K</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Selvax07</t>
+          <t>Senthamizh08</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1486,24 +1486,24 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/Selvax07/</t>
+          <t>https://leetcode.com/u/Senthamizh08/</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>922525106299</t>
+          <t>922525106300</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>SENTHAMIZHSELVAN K</t>
+          <t>Senthil.S</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Senthamizh08</t>
+          <t>Jna76WrjNd</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1513,24 +1513,24 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/Senthamizh08/</t>
+          <t>https://leetcode.com/u/Jna76WrjNd/</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>922525106300</t>
+          <t>922525106302</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Senthil.S</t>
+          <t>SHAHANA S</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Jna76WrjNd</t>
+          <t>shahana_pandiraj04</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -1540,24 +1540,24 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/Jna76WrjNd/</t>
+          <t>https://leetcode.com/u/shahana_pandiraj04/</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>922525106302</t>
+          <t>922525106303</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>SHAHANA S</t>
+          <t>SHANTHINI C</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>shahana_pandiraj04</t>
+          <t>ShanthiniChelladurai</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -1567,24 +1567,24 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/shahana_pandiraj04/</t>
+          <t>https://leetcode.com/u/ShanthiniChelladurai/</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>922525106303</t>
+          <t>922525106305</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>SHANTHINI C</t>
+          <t>SHARATH P</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>ShanthiniChelladurai</t>
+          <t>sharath_1010</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -1594,24 +1594,24 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/ShanthiniChelladurai/</t>
+          <t>https://leetcode.com/u/sharath_1010/</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>922525106305</t>
+          <t>922525106308</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>SHARATH P</t>
+          <t>SHREE HARINI L</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>sharath_1010</t>
+          <t>Shree_Harini478</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -1621,24 +1621,24 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/sharath_1010/</t>
+          <t>https://leetcode.com/u/Shree_Harini478/</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>922525106308</t>
+          <t>922525106310</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>SHREE HARINI L</t>
+          <t>SIVA MANIKANDAN K</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Shree_Harini478</t>
+          <t>9043374912</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -1648,24 +1648,24 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/Shree_Harini478/</t>
+          <t>https://leetcode.com/u/9043374912/</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>922525106310</t>
+          <t>922525106311</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>SIVA MANIKANDAN K</t>
+          <t>SIVA PRAKASH M</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>9043374912</t>
+          <t>sivaprakash_0406</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -1675,24 +1675,24 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/9043374912/</t>
+          <t>https://leetcode.com/u/sivaprakash_0406/</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>922525106311</t>
+          <t>922525106312</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>SIVA PRAKASH M</t>
+          <t>SIVADHARSHINI D</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>sivaprakash_0406</t>
+          <t>dharshinideivsigamani</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -1702,24 +1702,24 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/sivaprakash_0406/</t>
+          <t>https://leetcode.com/u/dharshinideivsigamani/</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>922525106312</t>
+          <t>922525106313</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>SIVADHARSHINI D</t>
+          <t>SIVAGNANAM M</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>dharshinideivsigamani</t>
+          <t>sivagnanam3344</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -1729,24 +1729,24 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/dharshinideivsigamani/</t>
+          <t>https://leetcode.com/u/sivagnanam3344/</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>922525106313</t>
+          <t>922525106315</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>SIVAGNANAM M</t>
+          <t>SIVANESH G</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>sivagnanam3344</t>
+          <t>GSIVANESH</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -1756,24 +1756,24 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/sivagnanam3344/</t>
+          <t>https://leetcode.com/u/GSIVANESH/</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>922525106315</t>
+          <t>922525106282</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>SIVANESH G</t>
+          <t>SANTHOSH PRIYAN S</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>GSIVANESH</t>
+          <t>8925787430</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -1783,24 +1783,24 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/GSIVANESH/</t>
+          <t>https://leetcode.com/u/8925787430/</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>922525106282</t>
+          <t>922525106280</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>SANTHOSH PRIYAN S</t>
+          <t>SANTHOSH D</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>8925787430</t>
+          <t>santhosh7811</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -1810,7 +1810,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/8925787430/</t>
+          <t>https://leetcode.com/u/santhosh7811/</t>
         </is>
       </c>
     </row>
@@ -1979,17 +1979,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>922525106366</t>
+          <t>922525106358</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>VIJAYARAGAVAN R</t>
+          <t>VASANTHA KUMAR D</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>vijayaragavan1216</t>
+          <t>Vasanthakumar12232</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -1999,24 +1999,24 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/vijayaragavan1216/</t>
+          <t>https://leetcode.com/u/Vasanthakumar12232/</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>922525106358</t>
+          <t>922525106352</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>VASANTHA KUMAR D</t>
+          <t>THIRINESH KUMAR S</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Vasanthakumar12232</t>
+          <t>THIRINESH KUMAR.S</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -2026,24 +2026,24 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/Vasanthakumar12232/</t>
+          <t>https://leetcode.com/u/THIRINESH KUMAR.S/</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>922525106352</t>
+          <t>922525106354</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>THIRINESH KUMAR S</t>
+          <t>THIRUMURUGAN S</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>THIRINESH KUMAR.S</t>
+          <t>thiru0211_</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -2053,24 +2053,24 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/THIRINESH KUMAR.S/</t>
+          <t>https://leetcode.com/u/thiru0211_/</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>922525106354</t>
+          <t>922525106355</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>THIRUMURUGAN S</t>
+          <t>VAISHNAVI U</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>thiru0211_</t>
+          <t>vaish200</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -2080,24 +2080,24 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/thiru0211_/</t>
+          <t>https://leetcode.com/u/vaish200/</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>922525106355</t>
+          <t>922525106356</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>VAISHNAVI U</t>
+          <t>VASANTH KUMAR C</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>vaish200</t>
+          <t>VASANTH2007</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -2107,24 +2107,24 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/vaish200/</t>
+          <t>https://leetcode.com/u/VASANTH2007/</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>922525106356</t>
+          <t>922525106357</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>VASANTH KUMAR C</t>
+          <t>VASANTH S</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>VASANTH2007</t>
+          <t>_vasanth_s_</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -2134,24 +2134,24 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/VASANTH2007/</t>
+          <t>https://leetcode.com/u/_vasanth_s_/</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>922525106357</t>
+          <t>922525106359</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>VASANTH S</t>
+          <t>VASANTHKUMAR R</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>_vasanth_s_</t>
+          <t>VasanthKumar008</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -2161,24 +2161,24 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/_vasanth_s_/</t>
+          <t>https://leetcode.com/u/VasanthKumar008/</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>922525106359</t>
+          <t>922525106366</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>VASANTHKUMAR R</t>
+          <t>VIJAYARAGAVAN R</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>VasanthKumar008</t>
+          <t>vijayaragavan1216</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -2188,7 +2188,7 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/VasanthKumar008/</t>
+          <t>https://leetcode.com/u/vijayaragavan1216/</t>
         </is>
       </c>
     </row>
@@ -2330,17 +2330,17 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>922525106372</t>
+          <t>922525106316</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>VISHWAJETH A M</t>
+          <t>SIVARANJAN M P</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>vishwajeth</t>
+          <t>SIVARANJAN_MP</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -2350,24 +2350,24 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/vishwajeth/</t>
+          <t>https://leetcode.com/u/SIVARANJAN_MP/</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>922525106316</t>
+          <t>922525106317</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>SIVARANJAN M P</t>
+          <t>SIVASANJEEV P</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>SIVARANJAN_MP</t>
+          <t>Sivasanjeev16</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -2377,24 +2377,24 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/SIVARANJAN_MP/</t>
+          <t>https://leetcode.com/u/Sivasanjeev16/</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>922525106317</t>
+          <t>922525106318</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>SIVASANJEEV P</t>
+          <t>SIVASUBRAMANI A</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Sivasanjeev16</t>
+          <t>AK_Siva</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -2404,24 +2404,24 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/Sivasanjeev16/</t>
+          <t>https://leetcode.com/u/AK_Siva/</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>922525106318</t>
+          <t>922525106319</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>SIVASUBRAMANI A</t>
+          <t>SIVATHARUN C</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>AK_Siva</t>
+          <t>sivatharun22</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -2431,24 +2431,24 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/AK_Siva/</t>
+          <t>https://leetcode.com/u/sivatharun22/</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>922525106319</t>
+          <t>922525106320</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>SIVATHARUN C</t>
+          <t>SOBIKA R</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>sivatharun22</t>
+          <t>_sobika_R</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -2458,24 +2458,24 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/sivatharun22/</t>
+          <t>https://leetcode.com/u/_sobika_R/</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>922525106320</t>
+          <t>922525106321</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>SOBIKA R</t>
+          <t>SREE DHARANI C</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>_sobika_R</t>
+          <t>SREEDHARANI_14</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -2485,24 +2485,24 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/_sobika_R/</t>
+          <t>https://leetcode.com/u/SREEDHARANI_14/</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>922525106321</t>
+          <t>922525106372</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>SREE DHARANI C</t>
+          <t>VISHWAJETH A M</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>SREEDHARANI_14</t>
+          <t>vishwajeth</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -2512,7 +2512,7 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/SREEDHARANI_14/</t>
+          <t>https://leetcode.com/u/vishwajeth/</t>
         </is>
       </c>
     </row>

</xml_diff>